<commit_message>
feat(world3): complete Station III and finalize World II transition
- finalize the World II to World III narrative transition
- integrate the complete Pixel Test Notebook experience
- add progressive index marks and interaction guides
- complete Plant, Prototype, Signal and Adjusted flows
- consolidate assets, responsive QA, tests and documentation
</commit_message>
<xml_diff>
--- a/docs/narrative/02_MATRIZ_DIALOGOS_Y_TEXTOS_GVO.xlsx
+++ b/docs/narrative/02_MATRIZ_DIALOGOS_Y_TEXTOS_GVO.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz" sheetId="1" r:id="R4601b69ae7054791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz" sheetId="1" r:id="Rd37d14bc75a847c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -85,9 +85,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -190,6 +190,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="12" max="12" width="50" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="72" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -1092,11 +1098,15 @@
       <x:c r="K22" t="str">
         <x:v>30-80 caracteres</x:v>
       </x:c>
-      <x:c r="L22" t="str"/>
+      <x:c r="L22" t="str">
+        <x:v>Abriendo Mundo III</x:v>
+      </x:c>
       <x:c r="M22" t="str"/>
-      <x:c r="N22" t="str"/>
+      <x:c r="N22" t="str">
+        <x:v>Copy runtime definitivo; aprobación humana consolidada por GVO-017K-R1.</x:v>
+      </x:c>
       <x:c r="O22" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>FINAL / human_approved</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1133,11 +1143,15 @@
       <x:c r="K23" t="str">
         <x:v>25-70 caracteres</x:v>
       </x:c>
-      <x:c r="L23" t="str"/>
+      <x:c r="L23" t="str">
+        <x:v>Preparando el Cuaderno Pixel de Pruebas…</x:v>
+      </x:c>
       <x:c r="M23" t="str"/>
-      <x:c r="N23" t="str"/>
+      <x:c r="N23" t="str">
+        <x:v>Copy runtime definitivo; aprobación humana consolidada por GVO-017K-R1.</x:v>
+      </x:c>
       <x:c r="O23" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>FINAL / human_approved</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -3556,7 +3570,7 @@
       <x:c r="M82" t="str"/>
       <x:c r="N82" t="str"/>
       <x:c r="O82" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -3597,7 +3611,7 @@
       <x:c r="M83" t="str"/>
       <x:c r="N83" t="str"/>
       <x:c r="O83" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -3638,7 +3652,7 @@
       <x:c r="M84" t="str"/>
       <x:c r="N84" t="str"/>
       <x:c r="O84" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -3679,7 +3693,7 @@
       <x:c r="M85" t="str"/>
       <x:c r="N85" t="str"/>
       <x:c r="O85" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -3720,7 +3734,7 @@
       <x:c r="M86" t="str"/>
       <x:c r="N86" t="str"/>
       <x:c r="O86" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -3761,7 +3775,7 @@
       <x:c r="M87" t="str"/>
       <x:c r="N87" t="str"/>
       <x:c r="O87" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -3802,7 +3816,7 @@
       <x:c r="M88" t="str"/>
       <x:c r="N88" t="str"/>
       <x:c r="O88" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -3843,7 +3857,7 @@
       <x:c r="M89" t="str"/>
       <x:c r="N89" t="str"/>
       <x:c r="O89" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -3884,7 +3898,7 @@
       <x:c r="M90" t="str"/>
       <x:c r="N90" t="str"/>
       <x:c r="O90" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -3925,7 +3939,7 @@
       <x:c r="M91" t="str"/>
       <x:c r="N91" t="str"/>
       <x:c r="O91" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -3966,7 +3980,7 @@
       <x:c r="M92" t="str"/>
       <x:c r="N92" t="str"/>
       <x:c r="O92" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -4007,7 +4021,7 @@
       <x:c r="M93" t="str"/>
       <x:c r="N93" t="str"/>
       <x:c r="O93" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4048,7 +4062,7 @@
       <x:c r="M94" t="str"/>
       <x:c r="N94" t="str"/>
       <x:c r="O94" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4089,7 +4103,7 @@
       <x:c r="M95" t="str"/>
       <x:c r="N95" t="str"/>
       <x:c r="O95" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -4130,7 +4144,7 @@
       <x:c r="M96" t="str"/>
       <x:c r="N96" t="str"/>
       <x:c r="O96" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -4171,7 +4185,7 @@
       <x:c r="M97" t="str"/>
       <x:c r="N97" t="str"/>
       <x:c r="O97" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4212,7 +4226,7 @@
       <x:c r="M98" t="str"/>
       <x:c r="N98" t="str"/>
       <x:c r="O98" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -4253,7 +4267,7 @@
       <x:c r="M99" t="str"/>
       <x:c r="N99" t="str"/>
       <x:c r="O99" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -4294,7 +4308,7 @@
       <x:c r="M100" t="str"/>
       <x:c r="N100" t="str"/>
       <x:c r="O100" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -4335,7 +4349,7 @@
       <x:c r="M101" t="str"/>
       <x:c r="N101" t="str"/>
       <x:c r="O101" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -4376,7 +4390,7 @@
       <x:c r="M102" t="str"/>
       <x:c r="N102" t="str"/>
       <x:c r="O102" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -4417,7 +4431,7 @@
       <x:c r="M103" t="str"/>
       <x:c r="N103" t="str"/>
       <x:c r="O103" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -4458,7 +4472,7 @@
       <x:c r="M104" t="str"/>
       <x:c r="N104" t="str"/>
       <x:c r="O104" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>LEGACY / no consumido por runtime</x:v>
       </x:c>
     </x:row>
     <x:row r="105">

</xml_diff>

<commit_message>
feat(final): publish approved editorial copy
</commit_message>
<xml_diff>
--- a/docs/narrative/02_MATRIZ_DIALOGOS_Y_TEXTOS_GVO.xlsx
+++ b/docs/narrative/02_MATRIZ_DIALOGOS_Y_TEXTOS_GVO.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz" sheetId="1" r:id="Rd37d14bc75a847c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz" sheetId="1" r:id="R5f3b1fd216be472b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7133,11 +7133,17 @@
       <x:c r="K169" t="str">
         <x:v>2-7 palabras</x:v>
       </x:c>
-      <x:c r="L169" t="str"/>
-      <x:c r="M169" t="str"/>
-      <x:c r="N169" t="str"/>
+      <x:c r="L169" t="str">
+        <x:v>Mirador final del jardín</x:v>
+      </x:c>
+      <x:c r="M169" t="str">
+        <x:v>Mirador final</x:v>
+      </x:c>
+      <x:c r="N169" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O169" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="170">
@@ -7174,11 +7180,17 @@
       <x:c r="K170" t="str">
         <x:v>2-8 palabras</x:v>
       </x:c>
-      <x:c r="L170" t="str"/>
-      <x:c r="M170" t="str"/>
-      <x:c r="N170" t="str"/>
+      <x:c r="L170" t="str">
+        <x:v>Recorrido completo</x:v>
+      </x:c>
+      <x:c r="M170" t="str">
+        <x:v>Recorrido completo</x:v>
+      </x:c>
+      <x:c r="N170" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O170" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -7215,11 +7227,17 @@
       <x:c r="K171" t="str">
         <x:v>90-170 caracteres</x:v>
       </x:c>
-      <x:c r="L171" t="str"/>
-      <x:c r="M171" t="str"/>
-      <x:c r="N171" t="str"/>
+      <x:c r="L171" t="str">
+        <x:v>Llegaste al final del recorrido. Puedes volver a cualquier mundo cuando quieras.</x:v>
+      </x:c>
+      <x:c r="M171" t="str">
+        <x:v>Cierre y revisión libre</x:v>
+      </x:c>
+      <x:c r="N171" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O171" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -7256,11 +7274,17 @@
       <x:c r="K172" t="str">
         <x:v>50-130 caracteres</x:v>
       </x:c>
-      <x:c r="L172" t="str"/>
-      <x:c r="M172" t="str"/>
-      <x:c r="N172" t="str"/>
+      <x:c r="L172" t="str">
+        <x:v>El jardín queda abierto para volver a mirarlo.</x:v>
+      </x:c>
+      <x:c r="M172" t="str">
+        <x:v>Jardín abierto</x:v>
+      </x:c>
+      <x:c r="N172" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O172" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -7297,11 +7321,17 @@
       <x:c r="K173" t="str">
         <x:v>2-6 palabras</x:v>
       </x:c>
-      <x:c r="L173" t="str"/>
-      <x:c r="M173" t="str"/>
-      <x:c r="N173" t="str"/>
+      <x:c r="L173" t="str">
+        <x:v>I — Raíz</x:v>
+      </x:c>
+      <x:c r="M173" t="str">
+        <x:v>I — Raíz</x:v>
+      </x:c>
+      <x:c r="N173" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O173" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="174">
@@ -7338,11 +7368,17 @@
       <x:c r="K174" t="str">
         <x:v>40-100 caracteres</x:v>
       </x:c>
-      <x:c r="L174" t="str"/>
-      <x:c r="M174" t="str"/>
-      <x:c r="N174" t="str"/>
+      <x:c r="L174" t="str">
+        <x:v>Reabriendo Mundo I: Raíz…</x:v>
+      </x:c>
+      <x:c r="M174" t="str">
+        <x:v>Reabrir Mundo I</x:v>
+      </x:c>
+      <x:c r="N174" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O174" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -7379,11 +7415,17 @@
       <x:c r="K175" t="str">
         <x:v>2-6 palabras</x:v>
       </x:c>
-      <x:c r="L175" t="str"/>
-      <x:c r="M175" t="str"/>
-      <x:c r="N175" t="str"/>
+      <x:c r="L175" t="str">
+        <x:v>II — Pulso invisible</x:v>
+      </x:c>
+      <x:c r="M175" t="str">
+        <x:v>II — Pulso invisible</x:v>
+      </x:c>
+      <x:c r="N175" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O175" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -7420,11 +7462,17 @@
       <x:c r="K176" t="str">
         <x:v>40-100 caracteres</x:v>
       </x:c>
-      <x:c r="L176" t="str"/>
-      <x:c r="M176" t="str"/>
-      <x:c r="N176" t="str"/>
+      <x:c r="L176" t="str">
+        <x:v>Reabriendo Mundo II: Pulso invisible…</x:v>
+      </x:c>
+      <x:c r="M176" t="str">
+        <x:v>Reabrir Mundo II</x:v>
+      </x:c>
+      <x:c r="N176" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O176" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -7461,11 +7509,17 @@
       <x:c r="K177" t="str">
         <x:v>2-6 palabras</x:v>
       </x:c>
-      <x:c r="L177" t="str"/>
-      <x:c r="M177" t="str"/>
-      <x:c r="N177" t="str"/>
+      <x:c r="L177" t="str">
+        <x:v>III — Cuaderno de pruebas</x:v>
+      </x:c>
+      <x:c r="M177" t="str">
+        <x:v>III — Cuaderno</x:v>
+      </x:c>
+      <x:c r="N177" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O177" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="178">
@@ -7502,11 +7556,17 @@
       <x:c r="K178" t="str">
         <x:v>40-100 caracteres</x:v>
       </x:c>
-      <x:c r="L178" t="str"/>
-      <x:c r="M178" t="str"/>
-      <x:c r="N178" t="str"/>
+      <x:c r="L178" t="str">
+        <x:v>Reabriendo Mundo III: Cuaderno de pruebas…</x:v>
+      </x:c>
+      <x:c r="M178" t="str">
+        <x:v>Reabrir Mundo III</x:v>
+      </x:c>
+      <x:c r="N178" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O178" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="179">
@@ -7543,11 +7603,17 @@
       <x:c r="K179" t="str">
         <x:v>2-6 palabras</x:v>
       </x:c>
-      <x:c r="L179" t="str"/>
-      <x:c r="M179" t="str"/>
-      <x:c r="N179" t="str"/>
+      <x:c r="L179" t="str">
+        <x:v>IV — Mesa de sistema</x:v>
+      </x:c>
+      <x:c r="M179" t="str">
+        <x:v>IV — Mesa</x:v>
+      </x:c>
+      <x:c r="N179" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O179" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="180">
@@ -7584,11 +7650,17 @@
       <x:c r="K180" t="str">
         <x:v>40-100 caracteres</x:v>
       </x:c>
-      <x:c r="L180" t="str"/>
-      <x:c r="M180" t="str"/>
-      <x:c r="N180" t="str"/>
+      <x:c r="L180" t="str">
+        <x:v>Reabriendo Mundo IV: Mesa de sistema…</x:v>
+      </x:c>
+      <x:c r="M180" t="str">
+        <x:v>Reabrir Mundo IV</x:v>
+      </x:c>
+      <x:c r="N180" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O180" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="181">
@@ -7625,11 +7697,17 @@
       <x:c r="K181" t="str">
         <x:v>2-6 palabras</x:v>
       </x:c>
-      <x:c r="L181" t="str"/>
-      <x:c r="M181" t="str"/>
-      <x:c r="N181" t="str"/>
+      <x:c r="L181" t="str">
+        <x:v>V — Mapa del presente</x:v>
+      </x:c>
+      <x:c r="M181" t="str">
+        <x:v>V — Mapa</x:v>
+      </x:c>
+      <x:c r="N181" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O181" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -7666,11 +7744,17 @@
       <x:c r="K182" t="str">
         <x:v>40-100 caracteres</x:v>
       </x:c>
-      <x:c r="L182" t="str"/>
-      <x:c r="M182" t="str"/>
-      <x:c r="N182" t="str"/>
+      <x:c r="L182" t="str">
+        <x:v>Reabriendo Mundo V: Mapa del presente…</x:v>
+      </x:c>
+      <x:c r="M182" t="str">
+        <x:v>Reabrir Mundo V</x:v>
+      </x:c>
+      <x:c r="N182" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O182" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -7707,11 +7791,17 @@
       <x:c r="K183" t="str">
         <x:v>60-130 caracteres</x:v>
       </x:c>
-      <x:c r="L183" t="str"/>
-      <x:c r="M183" t="str"/>
-      <x:c r="N183" t="str"/>
+      <x:c r="L183" t="str">
+        <x:v>Elige un mundo para revisarlo libremente.</x:v>
+      </x:c>
+      <x:c r="M183" t="str">
+        <x:v>Revisión libre</x:v>
+      </x:c>
+      <x:c r="N183" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O183" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -7748,11 +7838,17 @@
       <x:c r="K184" t="str">
         <x:v>1-4 palabras</x:v>
       </x:c>
-      <x:c r="L184" t="str"/>
-      <x:c r="M184" t="str"/>
-      <x:c r="N184" t="str"/>
+      <x:c r="L184" t="str">
+        <x:v>Volver al inicio</x:v>
+      </x:c>
+      <x:c r="M184" t="str">
+        <x:v>Volver al inicio</x:v>
+      </x:c>
+      <x:c r="N184" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O184" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
@@ -7789,11 +7885,17 @@
       <x:c r="K185" t="str">
         <x:v>50-120 caracteres</x:v>
       </x:c>
-      <x:c r="L185" t="str"/>
-      <x:c r="M185" t="str"/>
-      <x:c r="N185" t="str"/>
+      <x:c r="L185" t="str">
+        <x:v>Regresa a la portada sin borrar tu recorrido.</x:v>
+      </x:c>
+      <x:c r="M185" t="str">
+        <x:v>Conservar recorrido</x:v>
+      </x:c>
+      <x:c r="N185" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O185" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="186">
@@ -7830,11 +7932,17 @@
       <x:c r="K186" t="str">
         <x:v>1-4 palabras</x:v>
       </x:c>
-      <x:c r="L186" t="str"/>
-      <x:c r="M186" t="str"/>
-      <x:c r="N186" t="str"/>
+      <x:c r="L186" t="str">
+        <x:v>Reiniciar recorrido</x:v>
+      </x:c>
+      <x:c r="M186" t="str">
+        <x:v>Reiniciar recorrido</x:v>
+      </x:c>
+      <x:c r="N186" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O186" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -7871,11 +7979,17 @@
       <x:c r="K187" t="str">
         <x:v>60-130 caracteres</x:v>
       </x:c>
-      <x:c r="L187" t="str"/>
-      <x:c r="M187" t="str"/>
-      <x:c r="N187" t="str"/>
+      <x:c r="L187" t="str">
+        <x:v>¿Quieres reiniciar el recorrido completo? Volverás a comenzar desde el inicio.</x:v>
+      </x:c>
+      <x:c r="M187" t="str">
+        <x:v>Confirmar reinicio</x:v>
+      </x:c>
+      <x:c r="N187" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O187" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="188">
@@ -7912,11 +8026,17 @@
       <x:c r="K188" t="str">
         <x:v>1-3 palabras</x:v>
       </x:c>
-      <x:c r="L188" t="str"/>
-      <x:c r="M188" t="str"/>
-      <x:c r="N188" t="str"/>
+      <x:c r="L188" t="str">
+        <x:v>Cancelar</x:v>
+      </x:c>
+      <x:c r="M188" t="str">
+        <x:v>Cancelar</x:v>
+      </x:c>
+      <x:c r="N188" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O188" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="189">
@@ -7953,11 +8073,17 @@
       <x:c r="K189" t="str">
         <x:v>1-4 palabras</x:v>
       </x:c>
-      <x:c r="L189" t="str"/>
-      <x:c r="M189" t="str"/>
-      <x:c r="N189" t="str"/>
+      <x:c r="L189" t="str">
+        <x:v>Reiniciar recorrido</x:v>
+      </x:c>
+      <x:c r="M189" t="str">
+        <x:v>Reiniciar recorrido</x:v>
+      </x:c>
+      <x:c r="N189" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O189" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="190">
@@ -7994,11 +8120,18 @@
       <x:c r="K190" t="str">
         <x:v>Variable</x:v>
       </x:c>
-      <x:c r="L190" t="str"/>
-      <x:c r="M190" t="str"/>
-      <x:c r="N190" t="str"/>
+      <x:c r="L190" t="str">
+        <x:v>Desarrollado por Momotto S.A.S.
+A cargo del Ing. José David Pérez Zapata.</x:v>
+      </x:c>
+      <x:c r="M190" t="str">
+        <x:v>Créditos</x:v>
+      </x:c>
+      <x:c r="N190" t="str">
+        <x:v>Mostrar las dos líneas con salto DOM.</x:v>
+      </x:c>
       <x:c r="O190" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="191">
@@ -8035,11 +8168,17 @@
       <x:c r="K191" t="str">
         <x:v>90-180 caracteres</x:v>
       </x:c>
-      <x:c r="L191" t="str"/>
-      <x:c r="M191" t="str"/>
-      <x:c r="N191" t="str"/>
+      <x:c r="L191" t="str">
+        <x:v>Mirador final del jardín con cinco accesos de revisión, Lía, regreso a la portada y reinicio del recorrido.</x:v>
+      </x:c>
+      <x:c r="M191" t="str">
+        <x:v>Escena accesible final</x:v>
+      </x:c>
+      <x:c r="N191" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O191" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="192">
@@ -8076,11 +8215,17 @@
       <x:c r="K192" t="str">
         <x:v>50-110 caracteres</x:v>
       </x:c>
-      <x:c r="L192" t="str"/>
-      <x:c r="M192" t="str"/>
-      <x:c r="N192" t="str"/>
+      <x:c r="L192" t="str">
+        <x:v>Revisar Mundo I: Raíz</x:v>
+      </x:c>
+      <x:c r="M192" t="str">
+        <x:v>Revisar Mundo I</x:v>
+      </x:c>
+      <x:c r="N192" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O192" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="193">
@@ -8117,11 +8262,17 @@
       <x:c r="K193" t="str">
         <x:v>50-110 caracteres</x:v>
       </x:c>
-      <x:c r="L193" t="str"/>
-      <x:c r="M193" t="str"/>
-      <x:c r="N193" t="str"/>
+      <x:c r="L193" t="str">
+        <x:v>Revisar Mundo II: Pulso invisible</x:v>
+      </x:c>
+      <x:c r="M193" t="str">
+        <x:v>Revisar Mundo II</x:v>
+      </x:c>
+      <x:c r="N193" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O193" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="194">
@@ -8158,11 +8309,17 @@
       <x:c r="K194" t="str">
         <x:v>50-120 caracteres</x:v>
       </x:c>
-      <x:c r="L194" t="str"/>
-      <x:c r="M194" t="str"/>
-      <x:c r="N194" t="str"/>
+      <x:c r="L194" t="str">
+        <x:v>Revisar Mundo III: Cuaderno de pruebas</x:v>
+      </x:c>
+      <x:c r="M194" t="str">
+        <x:v>Revisar Mundo III</x:v>
+      </x:c>
+      <x:c r="N194" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O194" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="195">
@@ -8199,11 +8356,17 @@
       <x:c r="K195" t="str">
         <x:v>50-120 caracteres</x:v>
       </x:c>
-      <x:c r="L195" t="str"/>
-      <x:c r="M195" t="str"/>
-      <x:c r="N195" t="str"/>
+      <x:c r="L195" t="str">
+        <x:v>Revisar Mundo IV: Mesa de sistema</x:v>
+      </x:c>
+      <x:c r="M195" t="str">
+        <x:v>Revisar Mundo IV</x:v>
+      </x:c>
+      <x:c r="N195" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O195" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="196">
@@ -8240,11 +8403,17 @@
       <x:c r="K196" t="str">
         <x:v>50-120 caracteres</x:v>
       </x:c>
-      <x:c r="L196" t="str"/>
-      <x:c r="M196" t="str"/>
-      <x:c r="N196" t="str"/>
+      <x:c r="L196" t="str">
+        <x:v>Revisar Mundo V: Mapa del presente</x:v>
+      </x:c>
+      <x:c r="M196" t="str">
+        <x:v>Revisar Mundo V</x:v>
+      </x:c>
+      <x:c r="N196" t="str">
+        <x:v>Aprobado por Ing. José David; excepción de longitud aceptada.</x:v>
+      </x:c>
       <x:c r="O196" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
@@ -8281,11 +8450,17 @@
       <x:c r="K197" t="str">
         <x:v>50-120 caracteres</x:v>
       </x:c>
-      <x:c r="L197" t="str"/>
-      <x:c r="M197" t="str"/>
-      <x:c r="N197" t="str"/>
+      <x:c r="L197" t="str">
+        <x:v>Volver a la portada sin borrar el recorrido completado</x:v>
+      </x:c>
+      <x:c r="M197" t="str">
+        <x:v>Volver sin borrar</x:v>
+      </x:c>
+      <x:c r="N197" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O197" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
     <x:row r="198">
@@ -8322,11 +8497,252 @@
       <x:c r="K198" t="str">
         <x:v>50-130 caracteres</x:v>
       </x:c>
-      <x:c r="L198" t="str"/>
-      <x:c r="M198" t="str"/>
-      <x:c r="N198" t="str"/>
+      <x:c r="L198" t="str">
+        <x:v>Reiniciar el recorrido completo después de confirmar</x:v>
+      </x:c>
+      <x:c r="M198" t="str">
+        <x:v>Reinicio con confirmación</x:v>
+      </x:c>
+      <x:c r="N198" t="str">
+        <x:v>Aprobado por Ing. José David el 2026-08-04.</x:v>
+      </x:c>
       <x:c r="O198" t="str">
-        <x:v>Pendiente escritor</x:v>
+        <x:v>Aprobado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" t="str">
+        <x:v>FINAL_RETURN_TO_MIRADOR_BTN_01</x:v>
+      </x:c>
+      <x:c r="B199" t="str">
+        <x:v>Pantalla final — Mirador</x:v>
+      </x:c>
+      <x:c r="C199" t="str">
+        <x:v>final_return_to_mirador</x:v>
+      </x:c>
+      <x:c r="D199" t="str">
+        <x:v>Sistema / interfaz</x:v>
+      </x:c>
+      <x:c r="E199" t="str">
+        <x:v>Botón</x:v>
+      </x:c>
+      <x:c r="F199" t="str">
+        <x:v>Revisita de un mundo desde el Mirador.</x:v>
+      </x:c>
+      <x:c r="G199" t="str">
+        <x:v>Visitante revisita un mundo.</x:v>
+      </x:c>
+      <x:c r="H199" t="str">
+        <x:v>Volver al Mirador final.</x:v>
+      </x:c>
+      <x:c r="I199" t="str">
+        <x:v>Retorno al Mirador</x:v>
+      </x:c>
+      <x:c r="J199" t="str">
+        <x:v>Crear navegación sin ticket</x:v>
+      </x:c>
+      <x:c r="K199" t="str">
+        <x:v>1-4 palabras</x:v>
+      </x:c>
+      <x:c r="L199" t="str">
+        <x:v>Volver al Mirador</x:v>
+      </x:c>
+      <x:c r="M199" t="str">
+        <x:v>Volver al Mirador</x:v>
+      </x:c>
+      <x:c r="N199" t="str">
+        <x:v>Registrado sin consumidor funcional.</x:v>
+      </x:c>
+      <x:c r="O199" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" t="str">
+        <x:v>FINAL_ACCESSIBLE_RETURN_TO_MIRADOR_01</x:v>
+      </x:c>
+      <x:c r="B200" t="str">
+        <x:v>Pantalla final — Mirador</x:v>
+      </x:c>
+      <x:c r="C200" t="str">
+        <x:v>final_return_to_mirador</x:v>
+      </x:c>
+      <x:c r="D200" t="str">
+        <x:v>Sistema / accesibilidad</x:v>
+      </x:c>
+      <x:c r="E200" t="str">
+        <x:v>Nombre accesible</x:v>
+      </x:c>
+      <x:c r="F200" t="str">
+        <x:v>Revisita de un mundo desde el Mirador.</x:v>
+      </x:c>
+      <x:c r="G200" t="str">
+        <x:v>Visitante revisita un mundo.</x:v>
+      </x:c>
+      <x:c r="H200" t="str">
+        <x:v>Nombrar el retorno al Mirador.</x:v>
+      </x:c>
+      <x:c r="I200" t="str">
+        <x:v>Retorno accesible</x:v>
+      </x:c>
+      <x:c r="J200" t="str">
+        <x:v>Texto visible duplicado</x:v>
+      </x:c>
+      <x:c r="K200" t="str">
+        <x:v>Variable</x:v>
+      </x:c>
+      <x:c r="L200" t="str">
+        <x:v>Volver al Mirador final desde este mundo</x:v>
+      </x:c>
+      <x:c r="M200" t="str">
+        <x:v>Retorno accesible</x:v>
+      </x:c>
+      <x:c r="N200" t="str">
+        <x:v>Registrado sin consumidor funcional.</x:v>
+      </x:c>
+      <x:c r="O200" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" t="str">
+        <x:v>FINAL_RESTART_BUSY_01</x:v>
+      </x:c>
+      <x:c r="B201" t="str">
+        <x:v>Pantalla final — Mirador</x:v>
+      </x:c>
+      <x:c r="C201" t="str">
+        <x:v>final_restart_busy</x:v>
+      </x:c>
+      <x:c r="D201" t="str">
+        <x:v>Sistema</x:v>
+      </x:c>
+      <x:c r="E201" t="str">
+        <x:v>Estado busy</x:v>
+      </x:c>
+      <x:c r="F201" t="str">
+        <x:v>Reinicio completo en curso.</x:v>
+      </x:c>
+      <x:c r="G201" t="str">
+        <x:v>Visitante confirmó reinicio.</x:v>
+      </x:c>
+      <x:c r="H201" t="str">
+        <x:v>Anunciar reinicio en curso.</x:v>
+      </x:c>
+      <x:c r="I201" t="str">
+        <x:v>Reinicio en curso</x:v>
+      </x:c>
+      <x:c r="J201" t="str">
+        <x:v>Prometer éxito</x:v>
+      </x:c>
+      <x:c r="K201" t="str">
+        <x:v>Variable</x:v>
+      </x:c>
+      <x:c r="L201" t="str">
+        <x:v>Reiniciando recorrido…</x:v>
+      </x:c>
+      <x:c r="M201" t="str">
+        <x:v>Reiniciando</x:v>
+      </x:c>
+      <x:c r="N201" t="str">
+        <x:v>Registrado sin consumidor funcional.</x:v>
+      </x:c>
+      <x:c r="O201" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" t="str">
+        <x:v>FINAL_RESTART_ERROR_01</x:v>
+      </x:c>
+      <x:c r="B202" t="str">
+        <x:v>Pantalla final — Mirador</x:v>
+      </x:c>
+      <x:c r="C202" t="str">
+        <x:v>final_restart_error</x:v>
+      </x:c>
+      <x:c r="D202" t="str">
+        <x:v>Sistema</x:v>
+      </x:c>
+      <x:c r="E202" t="str">
+        <x:v>Error visible</x:v>
+      </x:c>
+      <x:c r="F202" t="str">
+        <x:v>Reinicio completo falló.</x:v>
+      </x:c>
+      <x:c r="G202" t="str">
+        <x:v>Fallo posterior a confirmación.</x:v>
+      </x:c>
+      <x:c r="H202" t="str">
+        <x:v>Informar fallo y conservación verificada.</x:v>
+      </x:c>
+      <x:c r="I202" t="str">
+        <x:v>Progreso conservado</x:v>
+      </x:c>
+      <x:c r="J202" t="str">
+        <x:v>Afirmar rollback no verificado</x:v>
+      </x:c>
+      <x:c r="K202" t="str">
+        <x:v>Variable</x:v>
+      </x:c>
+      <x:c r="L202" t="str">
+        <x:v>No pudimos reiniciar el recorrido. Tu progreso se conservó.</x:v>
+      </x:c>
+      <x:c r="M202" t="str">
+        <x:v>Error de reinicio</x:v>
+      </x:c>
+      <x:c r="N202" t="str">
+        <x:v>Solo consumir tras verificar rollback.</x:v>
+      </x:c>
+      <x:c r="O202" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" t="str">
+        <x:v>FINAL_RESTART_RETRY_BTN_01</x:v>
+      </x:c>
+      <x:c r="B203" t="str">
+        <x:v>Pantalla final — Mirador</x:v>
+      </x:c>
+      <x:c r="C203" t="str">
+        <x:v>final_restart_error</x:v>
+      </x:c>
+      <x:c r="D203" t="str">
+        <x:v>Sistema / interfaz</x:v>
+      </x:c>
+      <x:c r="E203" t="str">
+        <x:v>Botón</x:v>
+      </x:c>
+      <x:c r="F203" t="str">
+        <x:v>Error de reinicio visible.</x:v>
+      </x:c>
+      <x:c r="G203" t="str">
+        <x:v>Reinicio completo falló.</x:v>
+      </x:c>
+      <x:c r="H203" t="str">
+        <x:v>Reintentar la operación.</x:v>
+      </x:c>
+      <x:c r="I203" t="str">
+        <x:v>Reintento</x:v>
+      </x:c>
+      <x:c r="J203" t="str">
+        <x:v>Ejecutar sin confirmación</x:v>
+      </x:c>
+      <x:c r="K203" t="str">
+        <x:v>1-2 palabras</x:v>
+      </x:c>
+      <x:c r="L203" t="str">
+        <x:v>Reintentar</x:v>
+      </x:c>
+      <x:c r="M203" t="str">
+        <x:v>Reintentar</x:v>
+      </x:c>
+      <x:c r="N203" t="str">
+        <x:v>Registrado sin consumidor funcional.</x:v>
+      </x:c>
+      <x:c r="O203" t="str">
+        <x:v>Aprobado</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(final): publish responsive mirador composition
</commit_message>
<xml_diff>
--- a/docs/narrative/02_MATRIZ_DIALOGOS_Y_TEXTOS_GVO.xlsx
+++ b/docs/narrative/02_MATRIZ_DIALOGOS_Y_TEXTOS_GVO.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz" sheetId="1" r:id="R5f3b1fd216be472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz" sheetId="1" r:id="R37af3cd10dc54457"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8122,13 +8122,13 @@
       </x:c>
       <x:c r="L190" t="str">
         <x:v>Desarrollado por Momotto S.A.S.
-A cargo del Ing. José David Pérez Zapata.</x:v>
+A cargo del Ing. José David P. Z.</x:v>
       </x:c>
       <x:c r="M190" t="str">
         <x:v>Créditos</x:v>
       </x:c>
       <x:c r="N190" t="str">
-        <x:v>Mostrar las dos líneas con salto DOM.</x:v>
+        <x:v>Mostrar las dos líneas con salto DOM. Copy corto aprobado por GVO_FINAL_021K.</x:v>
       </x:c>
       <x:c r="O190" t="str">
         <x:v>Aprobado</x:v>

</xml_diff>